<commit_message>
fix bangladesh and bhutan
</commit_message>
<xml_diff>
--- a/inst/extdata/region/2026-08-10/wb_projects_gov_sar.xlsx
+++ b/inst/extdata/region/2026-08-10/wb_projects_gov_sar.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="73">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -195,9 +195,6 @@
     <t xml:space="preserve">8B</t>
   </si>
   <si>
-    <t xml:space="preserve">Bangladesh</t>
-  </si>
-  <si>
     <t xml:space="preserve">Analytical</t>
   </si>
   <si>
@@ -211,9 +208,6 @@
   </si>
   <si>
     <t xml:space="preserve">Rangeet Ghosh (ADM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bhutan</t>
   </si>
   <si>
     <t xml:space="preserve">P513759</t>
@@ -935,7 +929,7 @@
     <col min="3" max="3" width="60.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="10.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="12.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="36.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="17.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="10.71" hidden="0" customWidth="1"/>
@@ -1037,7 +1031,7 @@
         <v>59</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>60</v>
+        <v>27</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>2025</v>
@@ -1046,20 +1040,20 @@
         <v>45513</v>
       </c>
       <c r="I2" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J2" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="J2" s="2" t="s">
+      <c r="K2" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="K2" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="N2" s="2" t="s">
-        <v>65</v>
       </c>
       <c r="O2" s="2"/>
       <c r="P2" s="2"/>
@@ -1084,42 +1078,44 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3" s="2"/>
+        <v>66</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>67</v>
+      </c>
       <c r="D3" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>45513</v>
+        <v>45929</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>63</v>
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>64</v>
+        <v>43</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
@@ -1136,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="V3" s="2" t="s">
         <v>35</v>
@@ -1144,44 +1140,42 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>68</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>69</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="C4" s="2"/>
       <c r="D4" s="2" t="s">
         <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>71</v>
+        <v>40</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>45929</v>
+        <v>45513</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>43</v>
+        <v>63</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="O4" s="2"/>
       <c r="P4" s="2"/>
@@ -1198,7 +1192,7 @@
         <v>0</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="V4" s="2" t="s">
         <v>35</v>

</xml_diff>